<commit_message>
tudo pronto para o adulto SES
</commit_message>
<xml_diff>
--- a/Prestador/neotin/resultado/relatorio_neotin_APENAS_VALORES.xlsx
+++ b/Prestador/neotin/resultado/relatorio_neotin_APENAS_VALORES.xlsx
@@ -418,13 +418,13 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B1" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D1" t="n">
         <v>0</v>
@@ -436,7 +436,7 @@
         <v>0</v>
       </c>
       <c r="G1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H1" t="n">
         <v>0</v>
@@ -448,7 +448,7 @@
         <v>0</v>
       </c>
       <c r="K1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L1" t="n">
         <v>0</v>
@@ -468,7 +468,7 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -538,13 +538,13 @@
         <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
@@ -600,7 +600,7 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L5" t="n">
         <v>0</v>
@@ -608,25 +608,25 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -749,7 +749,7 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
@@ -781,7 +781,7 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
@@ -810,7 +810,7 @@
         <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
@@ -825,7 +825,7 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K11" t="n">
         <v>0</v>
@@ -962,7 +962,7 @@
         <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F15" t="n">
         <v>0</v>
@@ -988,37 +988,37 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" t="n">
         <v>13</v>
       </c>
-      <c r="C16" t="n">
-        <v>9</v>
-      </c>
       <c r="D16" t="n">
         <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F16" t="n">
         <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I16" t="n">
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L16" t="n">
         <v>0</v>

</xml_diff>